<commit_message>
Refocus LendAgent on commercial loan brokers; add lean team plan
- Subscribers are brokers: plans are now Solo Broker / Broker Team / Brokerage Firm
  ($499 / $1,499 / $3,999), priced at ~2% of expected broker commission
- State plainly that the business sells software only and never funds loans; capital
  figures relabeled as operating capital
- Agent prompt and documents reworked for broker workflow: lender-ready packages,
  term-sheet comparison, no lender choice or credit decisions
- Model: add lean founder-led team plan selector; results for both team plans

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Urr7hvPys7BEkpKegAU7wH
</commit_message>
<xml_diff>
--- a/lending-agent/model/LendAgent_Financial_Model.xlsx
+++ b/lending-agent/model/LendAgent_Financial_Model.xlsx
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="294">
   <si>
     <t xml:space="preserve">How to use this model</t>
   </si>
@@ -94,13 +94,13 @@
     <t xml:space="preserve">Pre-launch burn: all costs before first paid month</t>
   </si>
   <si>
-    <t xml:space="preserve">Peak capital required (deepest point of cumulative cash)</t>
+    <t xml:space="preserve">Peak operating capital needed (salaries, servers, marketing until profitable; no loan funding)</t>
   </si>
   <si>
     <t xml:space="preserve">Month of peak capital need</t>
   </si>
   <si>
-    <t xml:space="preserve">Recommended raise (peak need + 25% cushion)</t>
+    <t xml:space="preserve">Recommended funding for the business (peak need + 25% cushion)</t>
   </si>
   <si>
     <t xml:space="preserve">Monthly run-rate costs</t>
@@ -196,13 +196,13 @@
     <t xml:space="preserve">Pricing check</t>
   </si>
   <si>
-    <t xml:space="preserve">Starter price as % of expected commission</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Professional price as % of expected commission</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enterprise price as % of expected commission</t>
+    <t xml:space="preserve">Solo Broker price as % of expected commission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Broker Team price as % of expected commission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brokerage Firm price as % of expected commission</t>
   </si>
   <si>
     <t xml:space="preserve">Assumptions</t>
@@ -271,16 +271,16 @@
     <t xml:space="preserve">Plan mix (share of new accounts)</t>
   </si>
   <si>
-    <t xml:space="preserve">Starter (solo) share</t>
+    <t xml:space="preserve">Solo Broker plan share</t>
   </si>
   <si>
     <t xml:space="preserve">Assumption.</t>
   </si>
   <si>
-    <t xml:space="preserve">Professional (team) share</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enterprise (lender) share</t>
+    <t xml:space="preserve">Broker Team plan share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brokerage Firm plan share</t>
   </si>
   <si>
     <t xml:space="preserve">Assumption. Shares must total 100%.</t>
@@ -322,7 +322,7 @@
     <t xml:space="preserve">Base marketing spend per month ($), from 2 months pre-launch</t>
   </si>
   <si>
-    <t xml:space="preserve">Content, website, conferences (e.g. state broker associations, NAGGL, CREFC).</t>
+    <t xml:space="preserve">Content, website, broker conferences and associations (e.g. AACFB, state broker groups).</t>
   </si>
   <si>
     <t xml:space="preserve">Card/ACH processing as % of revenue</t>
@@ -373,6 +373,12 @@
     <t xml:space="preserve">After Type I.</t>
   </si>
   <si>
+    <t xml:space="preserve">Team plan: 1 = Full team, 2 = Lean founder-led team (see Staffing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lean = founder unpaid in year 1, fractional SME/security, later hires.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Other G&amp;A per month ($): software seats, travel, co-working</t>
   </si>
   <si>
@@ -388,25 +394,25 @@
     <t xml:space="preserve">Per account, per month</t>
   </si>
   <si>
-    <t xml:space="preserve">Starter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Professional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enterprise</t>
+    <t xml:space="preserve">Solo Broker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Broker Team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brokerage Firm</t>
   </si>
   <si>
     <t xml:space="preserve">Target subscriber</t>
   </si>
   <si>
-    <t xml:space="preserve">Solo broker / advisor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brokerage or advisory team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lender, bank, CU, large brokerage</t>
+    <t xml:space="preserve">Independent commercial loan broker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Broker with 2-3 partners or analysts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commercial brokerage firm (up to 10 brokers)</t>
   </si>
   <si>
     <t xml:space="preserve">Seats included</t>
@@ -415,7 +421,7 @@
     <t xml:space="preserve">Average loan size ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">Fee / commission (% of loan)</t>
+    <t xml:space="preserve">Broker fee / commission (% of loan)</t>
   </si>
   <si>
     <t xml:space="preserve">Loans closed per month</t>
@@ -427,7 +433,7 @@
     <t xml:space="preserve">Analyst hours saved per deal analyzed</t>
   </si>
   <si>
-    <t xml:space="preserve">Loaded analyst cost per hour ($)</t>
+    <t xml:space="preserve">Value of broker/analyst time per hour ($)</t>
   </si>
   <si>
     <t xml:space="preserve">Value of time saved per month ($)</t>
@@ -679,7 +685,7 @@
     <t xml:space="preserve">Observability / SIEM (e.g. Datadog)</t>
   </si>
   <si>
-    <t xml:space="preserve">Customer SSO/SCIM (e.g. WorkOS) for enterprise accounts</t>
+    <t xml:space="preserve">Single sign-on (e.g. WorkOS) for brokerage-firm accounts</t>
   </si>
   <si>
     <t xml:space="preserve">Support desk + in-app chat (Intercom / Zendesk)</t>
@@ -700,25 +706,31 @@
     <t xml:space="preserve">SaaS tooling total</t>
   </si>
   <si>
-    <t xml:space="preserve">Team plan (loaded monthly cost = salary x ~1.25 / 12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Support reps scale with accounts and are in COGS (see Assumptions).</t>
+    <t xml:space="preserve">Team plans (loaded monthly cost = salary x ~1.25 / 12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick the plan in Assumptions. Support reps scale with accounts and are in COGS.</t>
   </si>
   <si>
     <t xml:space="preserve">Role</t>
   </si>
   <si>
-    <t xml:space="preserve">Loaded $ / month</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Start month</t>
+    <t xml:space="preserve">Full: $ / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full: start month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lean: $ / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lean: start month</t>
   </si>
   <si>
     <t xml:space="preserve">Founder / CEO</t>
   </si>
   <si>
-    <t xml:space="preserve">Set to 0 if you will not draw a salary.</t>
+    <t xml:space="preserve">Lean: unpaid for the first 12 months.</t>
   </si>
   <si>
     <t xml:space="preserve">Founding AI / full-stack engineer</t>
@@ -730,16 +742,16 @@
     <t xml:space="preserve">Full-stack engineer</t>
   </si>
   <si>
-    <t xml:space="preserve">Commercial lending SME / product lead (fractional, then full-time)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ex-credit officer; writes policy templates, grades agent output.</t>
+    <t xml:space="preserve">Commercial lending SME / product lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ex-broker or credit officer; builds lender-ready package templates, grades agent output. Lean: half-time contractor.</t>
   </si>
   <si>
     <t xml:space="preserve">DevSecOps / security engineer</t>
   </si>
   <si>
-    <t xml:space="preserve">Owns SOC 2 controls + infra.</t>
+    <t xml:space="preserve">Owns SOC 2 controls + infra. Lean: fractional contractor.</t>
   </si>
   <si>
     <t xml:space="preserve">Account executive (base + commission)</t>
@@ -754,7 +766,7 @@
     <t xml:space="preserve">Compliance &amp; operations manager</t>
   </si>
   <si>
-    <t xml:space="preserve">Vendor DD questionnaires, audits.</t>
+    <t xml:space="preserve">Security questionnaires, audits.</t>
   </si>
   <si>
     <t xml:space="preserve">Account executive #2</t>
@@ -1514,94 +1526,94 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>14694.9</c:v>
+                  <c:v>11994</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>24640.5195</c:v>
+                  <c:v>21283.92</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>35162.5378725</c:v>
+                  <c:v>31108.7736</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>46312.5482944875</c:v>
+                  <c:v>41516.561988</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>58146.1343654293</c:v>
+                  <c:v>52558.99628454</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>70723.1927668619</c:v>
+                  <c:v>64291.7975913657</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>84108.2816491042</c:v>
+                  <c:v>76775.0209626359</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>98370.9968054035</c:v>
+                  <c:v>90073.4052145087</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>113586.377858597</c:v>
+                  <c:v>104256.75064216</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>129835.346863328</c:v>
+                  <c:v>119400.326878761</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>147205.181919036</c:v>
+                  <c:v>135585.313309659</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>165790.028596534</c:v>
+                  <c:v>152899.274648014</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>185691.452205133</c:v>
+                  <c:v>171436.674486598</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>207019.034169398</c:v>
+                  <c:v>191299.4298656</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>229891.016046108</c:v>
+                  <c:v>212597.510139421</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>254434.994994375</c:v>
+                  <c:v>235449.583688033</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>280788.67481689</c:v>
+                  <c:v>259983.716302097</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>309100.677019631</c:v>
+                  <c:v>286338.125377311</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>339531.416693157</c:v>
+                  <c:v>314661.994384266</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>372254.048402767</c:v>
+                  <c:v>345116.352437358</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>407455.487689791</c:v>
+                  <c:v>377875.024172139</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>445337.514234407</c:v>
+                  <c:v>413125.655557207</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>486117.963214356</c:v>
+                  <c:v>451070.821716798</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>530032.011916672</c:v>
+                  <c:v>491929.223326282</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>577333.569224043</c:v>
+                  <c:v>535936.97866772</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>628296.776207154</c:v>
+                  <c:v>583349.01899959</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>683217.626712783</c:v>
+                  <c:v>634440.595507049</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>742415.717548637</c:v>
+                  <c:v>689508.906760417</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>806236.138633888</c:v>
+                  <c:v>748874.856323734</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>875051.514313925</c:v>
+                  <c:v>812884.950926555</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1802,94 +1814,94 @@
                   <c:v>155250</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>149608.0626</c:v>
+                  <c:v>149529.7365</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>153327.151143</c:v>
+                  <c:v>153229.8097575</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>157302.505681065</c:v>
+                  <c:v>157184.946517163</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>172555.65902101</c:v>
+                  <c:v>172416.575418121</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>177109.840806013</c:v>
+                  <c:v>176947.813801667</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>181990.113907234</c:v>
+                  <c:v>181803.603447145</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>210223.521710634</c:v>
+                  <c:v>210010.857150727</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>215839.247171036</c:v>
+                  <c:v>215598.6170149</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>230368.784575181</c:v>
+                  <c:v>230098.225385904</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>261846.125030896</c:v>
+                  <c:v>261543.509451343</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>268807.956780825</c:v>
+                  <c:v>268470.980591153</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>276293.881527063</c:v>
+                  <c:v>275920.049662556</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>302346.648047905</c:v>
+                  <c:v>301933.259494067</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>319512.404490448</c:v>
+                  <c:v>319056.535965637</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>328840.970833426</c:v>
+                  <c:v>328339.459162132</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>338886.133134249</c:v>
+                  <c:v>338335.556206365</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>349705.961303284</c:v>
+                  <c:v>349102.617506355</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>369863.152287885</c:v>
+                  <c:v>369203.038290257</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>382425.400699245</c:v>
+                  <c:v>381704.187452287</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>395965.799077806</c:v>
+                  <c:v>395178.805894809</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>419063.270168586</c:v>
+                  <c:v>418205.436726574</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>434803.033767515</c:v>
+                  <c:v>433868.889865876</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>460277.110904721</c:v>
+                  <c:v>459260.743801292</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>478584.86835201</c:v>
+                  <c:v>477479.887482888</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>506833.606680708</c:v>
+                  <c:v>505633.105554575</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>528139.195354189</c:v>
+                  <c:v>526835.71039517</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>559626.758618073</c:v>
+                  <c:v>558212.224713107</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>584431.416252179</c:v>
+                  <c:v>582897.118739321</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>619699.083573397</c:v>
+                  <c:v>618035.606386403</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>657087.335429786</c:v>
+                  <c:v>655284.505091553</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1904,11 +1916,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="40488814"/>
-        <c:axId val="47171810"/>
+        <c:axId val="72057901"/>
+        <c:axId val="17069845"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="40488814"/>
+        <c:axId val="72057901"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1940,7 +1952,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47171810"/>
+        <c:crossAx val="17069845"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1948,7 +1960,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="47171810"/>
+        <c:axId val="17069845"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1990,7 +2002,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40488814"/>
+        <c:crossAx val="72057901"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2280,94 +2292,94 @@
                   <c:v>-739250</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-874163.1626</c:v>
+                  <c:v>-876785.7365</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-1002849.794243</c:v>
+                  <c:v>-1008731.6262575</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-1124989.76205157</c:v>
+                  <c:v>-1134807.79917466</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-1251232.87277809</c:v>
+                  <c:v>-1265707.81260478</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-1370196.57921867</c:v>
+                  <c:v>-1390096.63012191</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-1481463.50035904</c:v>
+                  <c:v>-1507608.43597769</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-1607578.74042057</c:v>
+                  <c:v>-1640844.27216578</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-1725046.99078621</c:v>
+                  <c:v>-1766369.48396617</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-1841829.39750279</c:v>
+                  <c:v>-1892210.95870992</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-1973840.17567036</c:v>
+                  <c:v>-2034354.1412825</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-2095442.95053215</c:v>
+                  <c:v>-2167239.80856399</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-2205946.80346267</c:v>
+                  <c:v>-2290260.58357853</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-2322601.99930545</c:v>
+                  <c:v>-2420757.168586</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-2435095.3696265</c:v>
+                  <c:v>-2548514.27468604</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-2534045.32441381</c:v>
+                  <c:v>-2664256.22370875</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-2618496.46255369</c:v>
+                  <c:v>-2767142.19622708</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-2687413.74904008</c:v>
+                  <c:v>-2856261.09743134</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-2748176.22430834</c:v>
+                  <c:v>-2939126.01034429</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-2791070.20831442</c:v>
+                  <c:v>-3006168.20341231</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-2814781.95898946</c:v>
+                  <c:v>-3056230.65686976</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-2826389.74146826</c:v>
+                  <c:v>-3096561.0694242</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-2815855.26100137</c:v>
+                  <c:v>-3117304.30373286</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-2790014.40869173</c:v>
+                  <c:v>-3125494.22581736</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-2738567.26512707</c:v>
+                  <c:v>-3111044.88997396</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-2668067.30258373</c:v>
+                  <c:v>-3080741.01686082</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-2567909.72173077</c:v>
+                  <c:v>-3024227.7082564</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-2444318.85363606</c:v>
+                  <c:v>-2947999.33746246</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-2286334.5523396</c:v>
+                  <c:v>-2841387.54944136</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-2099797.49727911</c:v>
+                  <c:v>-2710548.29950403</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-1881833.31839497</c:v>
+                  <c:v>-2552947.85366903</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2382,11 +2394,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="59019872"/>
-        <c:axId val="21203493"/>
+        <c:axId val="1655877"/>
+        <c:axId val="34257257"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="59019872"/>
+        <c:axId val="1655877"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2418,7 +2430,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21203493"/>
+        <c:crossAx val="34257257"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2426,7 +2438,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="21203493"/>
+        <c:axId val="34257257"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2468,7 +2480,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59019872"/>
+        <c:crossAx val="1655877"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2827,7 +2839,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="66"/>
@@ -2852,6 +2864,10 @@
         <f aca="false">Assumptions!$G$3</f>
         <v>Base</v>
       </c>
+      <c r="D3" s="2" t="str">
+        <f aca="false">IF(Assumptions!$F$34=1,"Full team","Lean team")</f>
+        <v>Full team</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -2882,7 +2898,7 @@
       </c>
       <c r="C8" s="7" t="n">
         <f aca="false">MAX(0,-MIN(Monthly!$C$39:$AL$39))</f>
-        <v>2826389.74146826</v>
+        <v>3125494.22581736</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2891,7 +2907,7 @@
       </c>
       <c r="C9" s="8" t="n">
         <f aca="false">INDEX(Monthly!$C$4:$AL$4,MATCH(MIN(Monthly!$C$39:$AL$39),Monthly!$C$39:$AL$39,0))</f>
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2900,7 +2916,7 @@
       </c>
       <c r="C10" s="7" t="n">
         <f aca="false">C8*1.25</f>
-        <v>3532987.17683532</v>
+        <v>3906867.7822717</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2932,7 +2948,7 @@
       </c>
       <c r="C14" s="6" t="n">
         <f aca="false">INDEX(Monthly!$C$40:$AL$40,12)</f>
-        <v>181990.113907234</v>
+        <v>181803.603447145</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2941,7 +2957,7 @@
       </c>
       <c r="C15" s="6" t="n">
         <f aca="false">INDEX(Monthly!$C$40:$AL$40,36)</f>
-        <v>657087.335429786</v>
+        <v>655284.505091553</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2955,7 +2971,7 @@
       </c>
       <c r="C17" s="6" t="n">
         <f aca="false">Pricing!$C$26</f>
-        <v>1499.15</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2982,7 +2998,7 @@
       </c>
       <c r="C20" s="6" t="n">
         <f aca="false">C17*(1-Assumptions!$F$26)-C18</f>
-        <v>1217.0229</v>
+        <v>1144.05225</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3000,7 +3016,7 @@
       </c>
       <c r="C22" s="6" t="n">
         <f aca="false">C20*C21</f>
-        <v>48680.916</v>
+        <v>45762.09</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3018,7 +3034,7 @@
       </c>
       <c r="C24" s="11" t="n">
         <f aca="false">IFERROR(C22/C23,0)</f>
-        <v>12.170229</v>
+        <v>11.4405225</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3027,7 +3043,7 @@
       </c>
       <c r="C25" s="10" t="n">
         <f aca="false">IFERROR(C23/C20,0)</f>
-        <v>3.28670890251942</v>
+        <v>3.49634380772382</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3041,7 +3057,7 @@
       </c>
       <c r="C27" s="12" t="n">
         <f aca="false">IF(MIN(Monthly!$C$42:$AL$42)=999,"Beyond month 36",MIN(Monthly!$C$42:$AL$42))</f>
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3086,7 +3102,7 @@
       </c>
       <c r="C32" s="7" t="n">
         <f aca="false">INDEX(Monthly!$C$14:$AL$14,36)*12</f>
-        <v>9863316.56879245</v>
+        <v>9368884.23037084</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3100,7 +3116,7 @@
       </c>
       <c r="C34" s="6" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,1,Monthly!$C$16:$AL$16)</f>
-        <v>249679.832799279</v>
+        <v>222754.049463906</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3109,7 +3125,7 @@
       </c>
       <c r="C35" s="6" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,2,Monthly!$C$16:$AL$16)</f>
-        <v>2205822.06294354</v>
+        <v>2036095.1315148</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3118,7 +3134,7 @@
       </c>
       <c r="C36" s="6" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,3,Monthly!$C$16:$AL$16)</f>
-        <v>6893279.78479158</v>
+        <v>6398774.37877912</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3127,7 +3143,7 @@
       </c>
       <c r="C37" s="6" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,1,Monthly!$C$38:$AL$38)</f>
-        <v>-1481463.50035904</v>
+        <v>-1507608.43597769</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3136,7 +3152,7 @@
       </c>
       <c r="C38" s="6" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,2,Monthly!$C$38:$AL$38)</f>
-        <v>-1266712.72394929</v>
+        <v>-1431517.5743666</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3145,7 +3161,7 @@
       </c>
       <c r="C39" s="6" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$AL$5,3,Monthly!$C$38:$AL$38)</f>
-        <v>866342.905913364</v>
+        <v>386178.156675261</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3154,7 +3170,7 @@
       </c>
       <c r="C40" s="13" t="n">
         <f aca="false">IFERROR(SUMIF(Monthly!$C$5:$AL$5,3,Monthly!$C$25:$AL$25)/SUMIF(Monthly!$C$5:$AL$5,3,Monthly!$C$16:$AL$16),0)</f>
-        <v>0.719241678513971</v>
+        <v>0.699785475870486</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3186,7 +3202,7 @@
       </c>
       <c r="C44" s="13" t="n">
         <f aca="false">Pricing!$E$16</f>
-        <v>0.0166666666666667</v>
+        <v>0.019995</v>
       </c>
     </row>
   </sheetData>
@@ -3206,7 +3222,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -3631,18 +3647,29 @@
       <c r="A34" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F34" s="19" t="n">
+      <c r="F34" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F35" s="19" t="n">
         <v>3000</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="G35" s="3" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F36" s="13" t="n">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F37" s="13" t="n">
         <f aca="false">Assumptions!$F$14+Assumptions!$F$15+Assumptions!$F$16</f>
         <v>1</v>
       </c>
@@ -3672,45 +3699,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C6" s="16" t="n">
         <v>1</v>
@@ -3724,7 +3751,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C7" s="19" t="n">
         <v>1500000</v>
@@ -3733,12 +3760,12 @@
         <v>2000000</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>3000000</v>
+        <v>2500000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C8" s="21" t="n">
         <v>0.01</v>
@@ -3747,12 +3774,12 @@
         <v>0.01</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>0.0075</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>1.5</v>
@@ -3761,12 +3788,12 @@
         <v>4</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C10" s="6" t="n">
         <f aca="false">C7*C8*C9</f>
@@ -3778,7 +3805,7 @@
       </c>
       <c r="E10" s="6" t="n">
         <f aca="false">E7*E8*E9</f>
-        <v>270000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3800,7 +3827,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>6</v>
@@ -3814,7 +3841,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C13" s="19" t="n">
         <v>75</v>
@@ -3823,12 +3850,12 @@
         <v>75</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C14" s="6" t="n">
         <f aca="false">C6*C11*C12*C13</f>
@@ -3840,12 +3867,12 @@
       </c>
       <c r="E14" s="6" t="n">
         <f aca="false">E6*E11*E12*E13</f>
-        <v>40800</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>499</v>
@@ -3854,12 +3881,12 @@
         <v>1499</v>
       </c>
       <c r="E15" s="23" t="n">
-        <v>4500</v>
+        <v>3999</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C16" s="13" t="n">
         <f aca="false">IFERROR(C15/C10,0)</f>
@@ -3871,12 +3898,12 @@
       </c>
       <c r="E16" s="13" t="n">
         <f aca="false">IFERROR(E15/E10,0)</f>
-        <v>0.0166666666666667</v>
+        <v>0.019995</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C17" s="11" t="n">
         <f aca="false">IFERROR(C14/C15,0)</f>
@@ -3888,12 +3915,12 @@
       </c>
       <c r="E17" s="11" t="n">
         <f aca="false">IFERROR(E14/E15,0)</f>
-        <v>9.06666666666667</v>
+        <v>9.00225056264066</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C18" s="6" t="n">
         <f aca="false">C10*$C$23</f>
@@ -3905,12 +3932,12 @@
       </c>
       <c r="E18" s="6" t="n">
         <f aca="false">E10*$C$23</f>
-        <v>8100</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C19" s="19" t="n">
         <v>0</v>
@@ -3919,12 +3946,12 @@
         <v>500</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>5000</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C20" s="24" t="n">
         <f aca="false">Assumptions!$F$14</f>
@@ -3941,7 +3968,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C23" s="25" t="n">
         <v>0.03</v>
@@ -3949,21 +3976,21 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C26" s="6" t="n">
         <f aca="false">SUMPRODUCT(C15:E15,C20:E20)</f>
-        <v>1499.15</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C27" s="10" t="n">
         <f aca="false">SUMPRODUCT(C6:E6,C20:E20)</f>
@@ -3972,16 +3999,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C28" s="6" t="n">
         <f aca="false">SUMPRODUCT(C19:E19,C20:E20)</f>
-        <v>950</v>
+        <v>575</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -4010,22 +4037,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>4</v>
@@ -4033,7 +4060,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C6" s="26" t="n">
         <v>20</v>
@@ -4041,7 +4068,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C7" s="26" t="n">
         <v>0.2</v>
@@ -4049,7 +4076,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C8" s="26" t="n">
         <v>2</v>
@@ -4057,7 +4084,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C9" s="26" t="n">
         <v>10</v>
@@ -4065,7 +4092,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C10" s="26" t="n">
         <v>0.2</v>
@@ -4073,7 +4100,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C11" s="26" t="n">
         <v>0.1</v>
@@ -4081,7 +4108,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C12" s="26" t="n">
         <v>0.5</v>
@@ -4089,7 +4116,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C13" s="27" t="n">
         <v>1.25</v>
@@ -4097,12 +4124,12 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C15" s="16" t="n">
         <v>250</v>
@@ -4110,7 +4137,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C16" s="16" t="n">
         <v>1500</v>
@@ -4118,7 +4145,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C17" s="16" t="n">
         <v>40000</v>
@@ -4126,7 +4153,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C18" s="9" t="n">
         <f aca="false">$C$15*$C$16/1000000*$C$11+$C$17/1000000*$C$12</f>
@@ -4135,12 +4162,12 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C20" s="16" t="n">
         <v>25</v>
@@ -4148,7 +4175,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C21" s="16" t="n">
         <v>120000</v>
@@ -4156,7 +4183,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C22" s="18" t="n">
         <v>0.85</v>
@@ -4164,7 +4191,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C23" s="16" t="n">
         <v>80000</v>
@@ -4172,7 +4199,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">$C$20*$C$21/1000000*($C$22*$C$7+(1-$C$22)*$C$5*$C$13)+$C$23/1000000*$C$6</f>
@@ -4181,12 +4208,12 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C26" s="18" t="n">
         <v>0.4</v>
@@ -4194,7 +4221,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C27" s="28" t="n">
         <v>0.015</v>
@@ -4202,7 +4229,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C28" s="9" t="n">
         <f aca="false">$C$15*$C$26*$C$27</f>
@@ -4211,12 +4238,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C30" s="16" t="n">
         <v>80</v>
@@ -4224,7 +4251,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C31" s="16" t="n">
         <v>60000</v>
@@ -4232,7 +4259,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C32" s="16" t="n">
         <v>4000</v>
@@ -4240,7 +4267,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C33" s="9" t="n">
         <f aca="false">$C$30*($C$31/1000000*($C$22*$C$10+(1-$C$22)*$C$8*$C$13)+$C$32/1000000*$C$9)</f>
@@ -4249,12 +4276,12 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C35" s="18" t="n">
         <v>0.25</v>
@@ -4262,7 +4289,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C36" s="9" t="n">
         <f aca="false">($C$18+$C$24)*(1+$C$35)</f>
@@ -4271,7 +4298,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C37" s="9" t="n">
         <f aca="false">$C$33*(1+$C$35)</f>
@@ -4304,127 +4331,127 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C5" s="19" t="n">
         <v>90</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C6" s="19" t="n">
         <v>240</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C7" s="19" t="n">
         <v>420</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C8" s="19" t="n">
         <v>150</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C9" s="19" t="n">
         <v>180</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C10" s="19" t="n">
         <v>90</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C11" s="19" t="n">
         <v>120</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C12" s="19" t="n">
         <v>40</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C13" s="19" t="n">
         <v>350</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C14" s="19" t="n">
         <v>250</v>
@@ -4433,18 +4460,18 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C15" s="19" t="n">
         <v>120</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C16" s="19" t="n">
         <v>600</v>
@@ -4453,18 +4480,18 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C17" s="19" t="n">
         <v>300</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C18" s="29" t="n">
         <f aca="false">SUM(C5:C17)</f>
@@ -4473,23 +4500,23 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C21" s="19" t="n">
         <v>1000</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C22" s="19" t="n">
         <v>900</v>
@@ -4498,7 +4525,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C23" s="19" t="n">
         <v>500</v>
@@ -4507,7 +4534,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C24" s="19" t="n">
         <v>400</v>
@@ -4516,7 +4543,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C25" s="19" t="n">
         <v>400</v>
@@ -4525,18 +4552,18 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C26" s="19" t="n">
         <v>300</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C27" s="19" t="n">
         <v>300</v>
@@ -4545,7 +4572,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C28" s="29" t="n">
         <f aca="false">SUM(C21:C27)</f>
@@ -4568,41 +4595,47 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>179</v>
+        <v>223</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C5" s="19" t="n">
         <v>12500</v>
@@ -4610,13 +4643,19 @@
       <c r="D5" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>222</v>
+      <c r="E5" s="19" t="n">
+        <v>12500</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C6" s="19" t="n">
         <v>22000</v>
@@ -4624,13 +4663,19 @@
       <c r="D6" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>224</v>
+      <c r="E6" s="19" t="n">
+        <v>22000</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C7" s="19" t="n">
         <v>18000</v>
@@ -4638,11 +4683,17 @@
       <c r="D7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="3"/>
+      <c r="E7" s="19" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="G7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="C8" s="19" t="n">
         <v>9000</v>
@@ -4650,13 +4701,19 @@
       <c r="D8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>227</v>
+      <c r="E8" s="19" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C9" s="19" t="n">
         <v>19000</v>
@@ -4664,13 +4721,19 @@
       <c r="D9" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>229</v>
+      <c r="E9" s="19" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C10" s="19" t="n">
         <v>13000</v>
@@ -4678,11 +4741,17 @@
       <c r="D10" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="E10" s="3"/>
+      <c r="E10" s="19" t="n">
+        <v>13000</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="C11" s="19" t="n">
         <v>11000</v>
@@ -4690,11 +4759,17 @@
       <c r="D11" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="E11" s="3"/>
+      <c r="E11" s="19" t="n">
+        <v>11000</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="G11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C12" s="19" t="n">
         <v>18000</v>
@@ -4702,11 +4777,17 @@
       <c r="D12" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="E12" s="3"/>
+      <c r="E12" s="19" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="G12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C13" s="19" t="n">
         <v>12000</v>
@@ -4714,13 +4795,19 @@
       <c r="D13" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>234</v>
+      <c r="E13" s="19" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="C14" s="19" t="n">
         <v>13000</v>
@@ -4728,11 +4815,17 @@
       <c r="D14" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="E14" s="3"/>
+      <c r="E14" s="19" t="n">
+        <v>13000</v>
+      </c>
+      <c r="F14" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C15" s="19" t="n">
         <v>18000</v>
@@ -4740,7 +4833,13 @@
       <c r="D15" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="E15" s="3"/>
+      <c r="E15" s="19" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="G15" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4767,28 +4866,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="C5" s="19" t="n">
         <v>6000</v>
@@ -4799,7 +4898,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C6" s="19" t="n">
         <v>25000</v>
@@ -4810,7 +4909,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C7" s="19" t="n">
         <v>12000</v>
@@ -4821,7 +4920,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="C8" s="19" t="n">
         <v>3000</v>
@@ -4832,7 +4931,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C9" s="19" t="n">
         <v>25000</v>
@@ -4843,7 +4942,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C10" s="19" t="n">
         <v>15000</v>
@@ -4854,7 +4953,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C11" s="19" t="n">
         <v>15000</v>
@@ -4865,7 +4964,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="C12" s="19" t="n">
         <v>15000</v>
@@ -4876,7 +4975,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C13" s="19" t="n">
         <v>15000</v>
@@ -4887,7 +4986,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="C14" s="19" t="n">
         <v>20000</v>
@@ -4898,7 +4997,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C15" s="19" t="n">
         <v>18000</v>
@@ -4909,7 +5008,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="C16" s="19" t="n">
         <v>15000</v>
@@ -4920,7 +5019,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B17" s="18" t="n">
         <v>0.15</v>
@@ -4935,7 +5034,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C18" s="29" t="n">
         <f aca="false">SUM(C5:C17)</f>
@@ -4968,17 +5067,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C4" s="30" t="n">
         <v>1</v>
@@ -5091,7 +5190,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C5" s="8" t="n">
         <f aca="false">ROUNDUP(C4/12,0)</f>
@@ -5240,7 +5339,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="2" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">IF(C4&gt;=Assumptions!$F$7,1,0)</f>
@@ -5389,7 +5488,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="2" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C8" s="10" t="n">
         <f aca="false">0</f>
@@ -5538,7 +5637,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="2" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="C9" s="10" t="n">
         <f aca="false">IF(C6=1,MIN(Assumptions!$F$11,Assumptions!$F$9*(1+Assumptions!$F$10)^(C4-Assumptions!$F$7)),0)</f>
@@ -5687,7 +5786,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="2" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C10" s="10" t="n">
         <f aca="false">C8*Assumptions!$F$12</f>
@@ -5836,7 +5935,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="14" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C11" s="31" t="n">
         <f aca="false">C8+C9-C10</f>
@@ -5985,7 +6084,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C12" s="10" t="n">
         <f aca="false">C11*Pricing!$C$27</f>
@@ -6134,7 +6233,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C14" s="6" t="n">
         <f aca="false">C11*Pricing!$C$26</f>
@@ -6162,128 +6261,128 @@
       </c>
       <c r="I14" s="6" t="n">
         <f aca="false">I11*Pricing!$C$26</f>
-        <v>8994.9</v>
+        <v>8544</v>
       </c>
       <c r="J14" s="6" t="n">
         <f aca="false">J11*Pricing!$C$26</f>
-        <v>18484.5195</v>
+        <v>17557.92</v>
       </c>
       <c r="K14" s="6" t="n">
         <f aca="false">K11*Pricing!$C$26</f>
-        <v>28514.0578725</v>
+        <v>27084.6936</v>
       </c>
       <c r="L14" s="6" t="n">
         <f aca="false">L11*Pricing!$C$26</f>
-        <v>39132.1898944875</v>
+        <v>37170.555588</v>
       </c>
       <c r="M14" s="6" t="n">
         <f aca="false">M11*Pricing!$C$26</f>
-        <v>50391.3472934293</v>
+        <v>47865.30937254</v>
       </c>
       <c r="N14" s="6" t="n">
         <f aca="false">N11*Pricing!$C$26</f>
-        <v>62348.0227291019</v>
+        <v>59222.6157264057</v>
       </c>
       <c r="O14" s="6" t="n">
         <f aca="false">O11*Pricing!$C$26</f>
-        <v>75063.0980083234</v>
+        <v>71300.3045484791</v>
       </c>
       <c r="P14" s="6" t="n">
         <f aca="false">P11*Pricing!$C$26</f>
-        <v>88602.1984733602</v>
+        <v>84160.7114872194</v>
       </c>
       <c r="Q14" s="6" t="n">
         <f aca="false">Q11*Pricing!$C$26</f>
-        <v>103036.075659991</v>
+        <v>97871.0414166873</v>
       </c>
       <c r="R14" s="6" t="n">
         <f aca="false">R11*Pricing!$C$26</f>
-        <v>118441.020488833</v>
+        <v>112503.76091525</v>
       </c>
       <c r="S14" s="6" t="n">
         <f aca="false">S11*Pricing!$C$26</f>
-        <v>134899.309434581</v>
+        <v>128137.022069068</v>
       </c>
       <c r="T14" s="6" t="n">
         <f aca="false">T11*Pricing!$C$26</f>
-        <v>152499.686313323</v>
+        <v>144855.120108176</v>
       </c>
       <c r="U14" s="6" t="n">
         <f aca="false">U11*Pricing!$C$26</f>
-        <v>171337.882539265</v>
+        <v>162748.987583573</v>
       </c>
       <c r="V14" s="6" t="n">
         <f aca="false">V11*Pricing!$C$26</f>
-        <v>191517.17893026</v>
+        <v>181916.728010333</v>
       </c>
       <c r="W14" s="6" t="n">
         <f aca="false">W11*Pricing!$C$26</f>
-        <v>213149.012387839</v>
+        <v>202464.192135732</v>
       </c>
       <c r="X14" s="6" t="n">
         <f aca="false">X11*Pricing!$C$26</f>
-        <v>236353.631043445</v>
+        <v>224505.600244049</v>
       </c>
       <c r="Y14" s="6" t="n">
         <f aca="false">Y11*Pricing!$C$26</f>
-        <v>261260.801749885</v>
+        <v>248164.214182594</v>
       </c>
       <c r="Z14" s="6" t="n">
         <f aca="false">Z11*Pricing!$C$26</f>
-        <v>288010.574107266</v>
+        <v>273573.063088248</v>
       </c>
       <c r="AA14" s="6" t="n">
         <f aca="false">AA11*Pricing!$C$26</f>
-        <v>316754.105547803</v>
+        <v>300875.727112078</v>
       </c>
       <c r="AB14" s="6" t="n">
         <f aca="false">AB11*Pricing!$C$26</f>
-        <v>347654.552365784</v>
+        <v>330227.183783395</v>
       </c>
       <c r="AC14" s="6" t="n">
         <f aca="false">AC11*Pricing!$C$26</f>
-        <v>380888.03196985</v>
+        <v>361794.722025859</v>
       </c>
       <c r="AD14" s="6" t="n">
         <f aca="false">AD11*Pricing!$C$26</f>
-        <v>416644.66205687</v>
+        <v>395758.929239225</v>
       </c>
       <c r="AE14" s="6" t="n">
         <f aca="false">AE11*Pricing!$C$26</f>
-        <v>455129.682862617</v>
+        <v>432314.757293377</v>
       </c>
       <c r="AF14" s="6" t="n">
         <f aca="false">AF11*Pricing!$C$26</f>
-        <v>496564.669136793</v>
+        <v>471672.673748987</v>
       </c>
       <c r="AG14" s="6" t="n">
         <f aca="false">AG11*Pricing!$C$26</f>
-        <v>541188.839021775</v>
+        <v>514059.905124242</v>
       </c>
       <c r="AH14" s="6" t="n">
         <f aca="false">AH11*Pricing!$C$26</f>
-        <v>589260.467588704</v>
+        <v>559721.779572634</v>
       </c>
       <c r="AI14" s="6" t="n">
         <f aca="false">AI11*Pricing!$C$26</f>
-        <v>641058.413404857</v>
+        <v>608923.176925936</v>
       </c>
       <c r="AJ14" s="6" t="n">
         <f aca="false">AJ11*Pricing!$C$26</f>
-        <v>696883.767176077</v>
+        <v>661950.094692815</v>
       </c>
       <c r="AK14" s="6" t="n">
         <f aca="false">AK11*Pricing!$C$26</f>
-        <v>757061.632231523</v>
+        <v>719111.339290724</v>
       </c>
       <c r="AL14" s="6" t="n">
         <f aca="false">AL11*Pricing!$C$26</f>
-        <v>821943.047399371</v>
+        <v>780740.352530903</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="C15" s="6" t="n">
         <f aca="false">C9*Pricing!$C$28</f>
@@ -6311,128 +6410,128 @@
       </c>
       <c r="I15" s="6" t="n">
         <f aca="false">I9*Pricing!$C$28</f>
-        <v>5700</v>
+        <v>3450</v>
       </c>
       <c r="J15" s="6" t="n">
         <f aca="false">J9*Pricing!$C$28</f>
-        <v>6156</v>
+        <v>3726</v>
       </c>
       <c r="K15" s="6" t="n">
         <f aca="false">K9*Pricing!$C$28</f>
-        <v>6648.48</v>
+        <v>4024.08</v>
       </c>
       <c r="L15" s="6" t="n">
         <f aca="false">L9*Pricing!$C$28</f>
-        <v>7180.3584</v>
+        <v>4346.0064</v>
       </c>
       <c r="M15" s="6" t="n">
         <f aca="false">M9*Pricing!$C$28</f>
-        <v>7754.787072</v>
+        <v>4693.686912</v>
       </c>
       <c r="N15" s="6" t="n">
         <f aca="false">N9*Pricing!$C$28</f>
-        <v>8375.17003776001</v>
+        <v>5069.18186496</v>
       </c>
       <c r="O15" s="6" t="n">
         <f aca="false">O9*Pricing!$C$28</f>
-        <v>9045.1836407808</v>
+        <v>5474.7164141568</v>
       </c>
       <c r="P15" s="6" t="n">
         <f aca="false">P9*Pricing!$C$28</f>
-        <v>9768.79833204327</v>
+        <v>5912.69372728935</v>
       </c>
       <c r="Q15" s="6" t="n">
         <f aca="false">Q9*Pricing!$C$28</f>
-        <v>10550.3021986067</v>
+        <v>6385.7092254725</v>
       </c>
       <c r="R15" s="6" t="n">
         <f aca="false">R9*Pricing!$C$28</f>
-        <v>11394.3263744953</v>
+        <v>6896.5659635103</v>
       </c>
       <c r="S15" s="6" t="n">
         <f aca="false">S9*Pricing!$C$28</f>
-        <v>12305.8724844549</v>
+        <v>7448.29124059112</v>
       </c>
       <c r="T15" s="6" t="n">
         <f aca="false">T9*Pricing!$C$28</f>
-        <v>13290.3422832113</v>
+        <v>8044.15453983841</v>
       </c>
       <c r="U15" s="6" t="n">
         <f aca="false">U9*Pricing!$C$28</f>
-        <v>14353.5696658682</v>
+        <v>8687.68690302548</v>
       </c>
       <c r="V15" s="6" t="n">
         <f aca="false">V9*Pricing!$C$28</f>
-        <v>15501.8552391376</v>
+        <v>9382.70185526752</v>
       </c>
       <c r="W15" s="6" t="n">
         <f aca="false">W9*Pricing!$C$28</f>
-        <v>16742.0036582687</v>
+        <v>10133.3180036889</v>
       </c>
       <c r="X15" s="6" t="n">
         <f aca="false">X9*Pricing!$C$28</f>
-        <v>18081.3639509302</v>
+        <v>10943.983443984</v>
       </c>
       <c r="Y15" s="6" t="n">
         <f aca="false">Y9*Pricing!$C$28</f>
-        <v>19527.8730670046</v>
+        <v>11819.5021195028</v>
       </c>
       <c r="Z15" s="6" t="n">
         <f aca="false">Z9*Pricing!$C$28</f>
-        <v>21090.1029123649</v>
+        <v>12765.062289063</v>
       </c>
       <c r="AA15" s="6" t="n">
         <f aca="false">AA9*Pricing!$C$28</f>
-        <v>22777.3111453541</v>
+        <v>13786.267272188</v>
       </c>
       <c r="AB15" s="6" t="n">
         <f aca="false">AB9*Pricing!$C$28</f>
-        <v>24599.4960369825</v>
+        <v>14889.1686539631</v>
       </c>
       <c r="AC15" s="6" t="n">
         <f aca="false">AC9*Pricing!$C$28</f>
-        <v>26567.4557199411</v>
+        <v>16080.3021462801</v>
       </c>
       <c r="AD15" s="6" t="n">
         <f aca="false">AD9*Pricing!$C$28</f>
-        <v>28692.8521775363</v>
+        <v>17366.7263179825</v>
       </c>
       <c r="AE15" s="6" t="n">
         <f aca="false">AE9*Pricing!$C$28</f>
-        <v>30988.2803517393</v>
+        <v>18756.0644234211</v>
       </c>
       <c r="AF15" s="6" t="n">
         <f aca="false">AF9*Pricing!$C$28</f>
-        <v>33467.3427798784</v>
+        <v>20256.5495772948</v>
       </c>
       <c r="AG15" s="6" t="n">
         <f aca="false">AG9*Pricing!$C$28</f>
-        <v>36144.7302022687</v>
+        <v>21877.0735434784</v>
       </c>
       <c r="AH15" s="6" t="n">
         <f aca="false">AH9*Pricing!$C$28</f>
-        <v>39036.3086184502</v>
+        <v>23627.2394269567</v>
       </c>
       <c r="AI15" s="6" t="n">
         <f aca="false">AI9*Pricing!$C$28</f>
-        <v>42159.2133079262</v>
+        <v>25517.4185811132</v>
       </c>
       <c r="AJ15" s="6" t="n">
         <f aca="false">AJ9*Pricing!$C$28</f>
-        <v>45531.9503725603</v>
+        <v>27558.8120676023</v>
       </c>
       <c r="AK15" s="6" t="n">
         <f aca="false">AK9*Pricing!$C$28</f>
-        <v>49174.5064023651</v>
+        <v>29763.5170330105</v>
       </c>
       <c r="AL15" s="6" t="n">
         <f aca="false">AL9*Pricing!$C$28</f>
-        <v>53108.4669145543</v>
+        <v>32144.5983956513</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="14" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C16" s="29" t="n">
         <f aca="false">C14+C15</f>
@@ -6460,128 +6559,128 @@
       </c>
       <c r="I16" s="29" t="n">
         <f aca="false">I14+I15</f>
-        <v>14694.9</v>
+        <v>11994</v>
       </c>
       <c r="J16" s="29" t="n">
         <f aca="false">J14+J15</f>
-        <v>24640.5195</v>
+        <v>21283.92</v>
       </c>
       <c r="K16" s="29" t="n">
         <f aca="false">K14+K15</f>
-        <v>35162.5378725</v>
+        <v>31108.7736</v>
       </c>
       <c r="L16" s="29" t="n">
         <f aca="false">L14+L15</f>
-        <v>46312.5482944875</v>
+        <v>41516.561988</v>
       </c>
       <c r="M16" s="29" t="n">
         <f aca="false">M14+M15</f>
-        <v>58146.1343654293</v>
+        <v>52558.99628454</v>
       </c>
       <c r="N16" s="29" t="n">
         <f aca="false">N14+N15</f>
-        <v>70723.1927668619</v>
+        <v>64291.7975913657</v>
       </c>
       <c r="O16" s="29" t="n">
         <f aca="false">O14+O15</f>
-        <v>84108.2816491042</v>
+        <v>76775.0209626359</v>
       </c>
       <c r="P16" s="29" t="n">
         <f aca="false">P14+P15</f>
-        <v>98370.9968054035</v>
+        <v>90073.4052145087</v>
       </c>
       <c r="Q16" s="29" t="n">
         <f aca="false">Q14+Q15</f>
-        <v>113586.377858597</v>
+        <v>104256.75064216</v>
       </c>
       <c r="R16" s="29" t="n">
         <f aca="false">R14+R15</f>
-        <v>129835.346863328</v>
+        <v>119400.326878761</v>
       </c>
       <c r="S16" s="29" t="n">
         <f aca="false">S14+S15</f>
-        <v>147205.181919036</v>
+        <v>135585.313309659</v>
       </c>
       <c r="T16" s="29" t="n">
         <f aca="false">T14+T15</f>
-        <v>165790.028596534</v>
+        <v>152899.274648014</v>
       </c>
       <c r="U16" s="29" t="n">
         <f aca="false">U14+U15</f>
-        <v>185691.452205133</v>
+        <v>171436.674486598</v>
       </c>
       <c r="V16" s="29" t="n">
         <f aca="false">V14+V15</f>
-        <v>207019.034169398</v>
+        <v>191299.4298656</v>
       </c>
       <c r="W16" s="29" t="n">
         <f aca="false">W14+W15</f>
-        <v>229891.016046108</v>
+        <v>212597.510139421</v>
       </c>
       <c r="X16" s="29" t="n">
         <f aca="false">X14+X15</f>
-        <v>254434.994994375</v>
+        <v>235449.583688033</v>
       </c>
       <c r="Y16" s="29" t="n">
         <f aca="false">Y14+Y15</f>
-        <v>280788.67481689</v>
+        <v>259983.716302097</v>
       </c>
       <c r="Z16" s="29" t="n">
         <f aca="false">Z14+Z15</f>
-        <v>309100.677019631</v>
+        <v>286338.125377311</v>
       </c>
       <c r="AA16" s="29" t="n">
         <f aca="false">AA14+AA15</f>
-        <v>339531.416693157</v>
+        <v>314661.994384266</v>
       </c>
       <c r="AB16" s="29" t="n">
         <f aca="false">AB14+AB15</f>
-        <v>372254.048402767</v>
+        <v>345116.352437358</v>
       </c>
       <c r="AC16" s="29" t="n">
         <f aca="false">AC14+AC15</f>
-        <v>407455.487689791</v>
+        <v>377875.024172139</v>
       </c>
       <c r="AD16" s="29" t="n">
         <f aca="false">AD14+AD15</f>
-        <v>445337.514234407</v>
+        <v>413125.655557207</v>
       </c>
       <c r="AE16" s="29" t="n">
         <f aca="false">AE14+AE15</f>
-        <v>486117.963214356</v>
+        <v>451070.821716798</v>
       </c>
       <c r="AF16" s="29" t="n">
         <f aca="false">AF14+AF15</f>
-        <v>530032.011916672</v>
+        <v>491929.223326282</v>
       </c>
       <c r="AG16" s="29" t="n">
         <f aca="false">AG14+AG15</f>
-        <v>577333.569224043</v>
+        <v>535936.97866772</v>
       </c>
       <c r="AH16" s="29" t="n">
         <f aca="false">AH14+AH15</f>
-        <v>628296.776207154</v>
+        <v>583349.01899959</v>
       </c>
       <c r="AI16" s="29" t="n">
         <f aca="false">AI14+AI15</f>
-        <v>683217.626712783</v>
+        <v>634440.595507049</v>
       </c>
       <c r="AJ16" s="29" t="n">
         <f aca="false">AJ14+AJ15</f>
-        <v>742415.717548637</v>
+        <v>689508.906760417</v>
       </c>
       <c r="AK16" s="29" t="n">
         <f aca="false">AK14+AK15</f>
-        <v>806236.138633888</v>
+        <v>748874.856323734</v>
       </c>
       <c r="AL16" s="29" t="n">
         <f aca="false">AL14+AL15</f>
-        <v>875051.514313925</v>
+        <v>812884.950926555</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="2" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C18" s="6" t="n">
         <f aca="false">C12*(Assumptions!$F$18*UnitCosts!$C$36+UnitCosts!$C$37)</f>
@@ -6730,7 +6829,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C19" s="6" t="n">
         <f aca="false">C12*Assumptions!$F$18*UnitCosts!$C$28</f>
@@ -6879,7 +6978,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="C20" s="6" t="n">
         <f aca="false">IF(C4&gt;=Assumptions!$F$7-1,Infrastructure!$C$18,Infrastructure!$C$18*Assumptions!$F$29)</f>
@@ -7028,7 +7127,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C21" s="6" t="n">
         <f aca="false">C12*Assumptions!$F$27+C11*Assumptions!$F$28</f>
@@ -7177,7 +7276,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C22" s="6" t="n">
         <f aca="false">C16*Assumptions!$F$26</f>
@@ -7205,128 +7304,128 @@
       </c>
       <c r="I22" s="6" t="n">
         <f aca="false">I16*Assumptions!$F$26</f>
-        <v>426.1521</v>
+        <v>347.826</v>
       </c>
       <c r="J22" s="6" t="n">
         <f aca="false">J16*Assumptions!$F$26</f>
-        <v>714.5750655</v>
+        <v>617.23368</v>
       </c>
       <c r="K22" s="6" t="n">
         <f aca="false">K16*Assumptions!$F$26</f>
-        <v>1019.7135983025</v>
+        <v>902.1544344</v>
       </c>
       <c r="L22" s="6" t="n">
         <f aca="false">L16*Assumptions!$F$26</f>
-        <v>1343.06390054014</v>
+        <v>1203.980297652</v>
       </c>
       <c r="M22" s="6" t="n">
         <f aca="false">M16*Assumptions!$F$26</f>
-        <v>1686.23789659745</v>
+        <v>1524.21089225166</v>
       </c>
       <c r="N22" s="6" t="n">
         <f aca="false">N16*Assumptions!$F$26</f>
-        <v>2050.972590239</v>
+        <v>1864.46213014961</v>
       </c>
       <c r="O22" s="6" t="n">
         <f aca="false">O16*Assumptions!$F$26</f>
-        <v>2439.14016782402</v>
+        <v>2226.47560791644</v>
       </c>
       <c r="P22" s="6" t="n">
         <f aca="false">P16*Assumptions!$F$26</f>
-        <v>2852.7589073567</v>
+        <v>2612.12875122075</v>
       </c>
       <c r="Q22" s="6" t="n">
         <f aca="false">Q16*Assumptions!$F$26</f>
-        <v>3294.00495789933</v>
+        <v>3023.44576862263</v>
       </c>
       <c r="R22" s="6" t="n">
         <f aca="false">R16*Assumptions!$F$26</f>
-        <v>3765.22505903651</v>
+        <v>3462.60947948406</v>
       </c>
       <c r="S22" s="6" t="n">
         <f aca="false">S16*Assumptions!$F$26</f>
-        <v>4268.95027565204</v>
+        <v>3931.97408598011</v>
       </c>
       <c r="T22" s="6" t="n">
         <f aca="false">T16*Assumptions!$F$26</f>
-        <v>4807.91082929949</v>
+        <v>4434.07896479241</v>
       </c>
       <c r="U22" s="6" t="n">
         <f aca="false">U16*Assumptions!$F$26</f>
-        <v>5385.05211394886</v>
+        <v>4971.66356011135</v>
       </c>
       <c r="V22" s="6" t="n">
         <f aca="false">V16*Assumptions!$F$26</f>
-        <v>6003.55199091254</v>
+        <v>5547.68346610241</v>
       </c>
       <c r="W22" s="6" t="n">
         <f aca="false">W16*Assumptions!$F$26</f>
-        <v>6666.83946533712</v>
+        <v>6165.32779404321</v>
       </c>
       <c r="X22" s="6" t="n">
         <f aca="false">X16*Assumptions!$F$26</f>
-        <v>7378.61485483688</v>
+        <v>6828.03792695295</v>
       </c>
       <c r="Y22" s="6" t="n">
         <f aca="false">Y16*Assumptions!$F$26</f>
-        <v>8142.8715696898</v>
+        <v>7539.52777276081</v>
       </c>
       <c r="Z22" s="6" t="n">
         <f aca="false">Z16*Assumptions!$F$26</f>
-        <v>8963.9196335693</v>
+        <v>8303.80563594202</v>
       </c>
       <c r="AA22" s="6" t="n">
         <f aca="false">AA16*Assumptions!$F$26</f>
-        <v>9846.41108410156</v>
+        <v>9125.19783714371</v>
       </c>
       <c r="AB22" s="6" t="n">
         <f aca="false">AB16*Assumptions!$F$26</f>
-        <v>10795.3674036802</v>
+        <v>10008.3742206834</v>
       </c>
       <c r="AC22" s="6" t="n">
         <f aca="false">AC16*Assumptions!$F$26</f>
-        <v>11816.2091430039</v>
+        <v>10958.375700992</v>
       </c>
       <c r="AD22" s="6" t="n">
         <f aca="false">AD16*Assumptions!$F$26</f>
-        <v>12914.7879127978</v>
+        <v>11980.644011159</v>
       </c>
       <c r="AE22" s="6" t="n">
         <f aca="false">AE16*Assumptions!$F$26</f>
-        <v>14097.4209332163</v>
+        <v>13081.0538297872</v>
       </c>
       <c r="AF22" s="6" t="n">
         <f aca="false">AF16*Assumptions!$F$26</f>
-        <v>15370.9283455835</v>
+        <v>14265.9474764622</v>
       </c>
       <c r="AG22" s="6" t="n">
         <f aca="false">AG16*Assumptions!$F$26</f>
-        <v>16742.6735074973</v>
+        <v>15542.1723813639</v>
       </c>
       <c r="AH22" s="6" t="n">
         <f aca="false">AH16*Assumptions!$F$26</f>
-        <v>18220.6065100075</v>
+        <v>16917.1215509881</v>
       </c>
       <c r="AI22" s="6" t="n">
         <f aca="false">AI16*Assumptions!$F$26</f>
-        <v>19813.3111746707</v>
+        <v>18398.7772697044</v>
       </c>
       <c r="AJ22" s="6" t="n">
         <f aca="false">AJ16*Assumptions!$F$26</f>
-        <v>21530.0558089105</v>
+        <v>19995.7582960521</v>
       </c>
       <c r="AK22" s="6" t="n">
         <f aca="false">AK16*Assumptions!$F$26</f>
-        <v>23380.8480203827</v>
+        <v>21717.3708333883</v>
       </c>
       <c r="AL22" s="6" t="n">
         <f aca="false">AL16*Assumptions!$F$26</f>
-        <v>25376.4939151038</v>
+        <v>23573.6635768701</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="C23" s="6" t="n">
         <f aca="false">IF(C6=1,MAX(1,ROUNDUP(C11/Assumptions!$F$20,0))*Assumptions!$F$24,0)</f>
@@ -7475,7 +7574,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="14" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="C24" s="29" t="n">
         <f aca="false">SUM(C18:C23)</f>
@@ -7503,128 +7602,128 @@
       </c>
       <c r="I24" s="29" t="n">
         <f aca="false">SUM(I18:I23)</f>
-        <v>13308.0626</v>
+        <v>13229.7365</v>
       </c>
       <c r="J24" s="29" t="n">
         <f aca="false">SUM(J18:J23)</f>
-        <v>15107.151143</v>
+        <v>15009.8097575</v>
       </c>
       <c r="K24" s="29" t="n">
         <f aca="false">SUM(K18:K23)</f>
-        <v>17008.905681065</v>
+        <v>16891.3465171625</v>
       </c>
       <c r="L24" s="29" t="n">
         <f aca="false">SUM(L18:L23)</f>
-        <v>19022.5710210096</v>
+        <v>18883.4874181214</v>
       </c>
       <c r="M24" s="29" t="n">
         <f aca="false">SUM(M18:M23)</f>
-        <v>21158.1057660132</v>
+        <v>20996.0787616674</v>
       </c>
       <c r="N24" s="29" t="n">
         <f aca="false">SUM(N18:N23)</f>
-        <v>23426.2400640341</v>
+        <v>23239.7296039447</v>
       </c>
       <c r="O24" s="29" t="n">
         <f aca="false">SUM(O18:O23)</f>
-        <v>25838.5379599782</v>
+        <v>25625.8734000706</v>
       </c>
       <c r="P24" s="29" t="n">
         <f aca="false">SUM(P18:P23)</f>
-        <v>28407.4647203272</v>
+        <v>28166.8345641913</v>
       </c>
       <c r="Q24" s="29" t="n">
         <f aca="false">SUM(Q18:Q23)</f>
-        <v>39646.4595284154</v>
+        <v>39375.9003391387</v>
       </c>
       <c r="R24" s="29" t="n">
         <f aca="false">SUM(R18:R23)</f>
-        <v>42570.0139803891</v>
+        <v>42267.3984008367</v>
       </c>
       <c r="S24" s="29" t="n">
         <f aca="false">SUM(S18:S23)</f>
-        <v>45693.7568462782</v>
+        <v>45356.7806566063</v>
       </c>
       <c r="T24" s="29" t="n">
         <f aca="false">SUM(T18:T23)</f>
-        <v>49034.545597752</v>
+        <v>48660.7137332449</v>
       </c>
       <c r="U24" s="29" t="n">
         <f aca="false">SUM(U18:U23)</f>
-        <v>52610.5652442494</v>
+        <v>52197.1766904118</v>
       </c>
       <c r="V24" s="29" t="n">
         <f aca="false">SUM(V18:V23)</f>
-        <v>64941.4350624996</v>
+        <v>64485.5665376895</v>
       </c>
       <c r="W24" s="29" t="n">
         <f aca="false">SUM(W18:W23)</f>
-        <v>69048.3238512421</v>
+        <v>68546.8121799482</v>
       </c>
       <c r="X24" s="29" t="n">
         <f aca="false">SUM(X18:X23)</f>
-        <v>73454.0743934904</v>
+        <v>72903.4974656065</v>
       </c>
       <c r="Y24" s="29" t="n">
         <f aca="false">SUM(Y18:Y23)</f>
-        <v>78183.3378632649</v>
+        <v>77579.9940663359</v>
       </c>
       <c r="Z24" s="29" t="n">
         <f aca="false">SUM(Z18:Z23)</f>
-        <v>91762.718972664</v>
+        <v>91102.6049750367</v>
       </c>
       <c r="AA24" s="29" t="n">
         <f aca="false">SUM(AA18:AA23)</f>
-        <v>97220.9327188065</v>
+        <v>96499.7194718487</v>
       </c>
       <c r="AB24" s="29" t="n">
         <f aca="false">SUM(AB18:AB23)</f>
-        <v>103088.973658932</v>
+        <v>102301.980475935</v>
       </c>
       <c r="AC24" s="29" t="n">
         <f aca="false">SUM(AC18:AC23)</f>
-        <v>117900.298716202</v>
+        <v>117042.465274191</v>
       </c>
       <c r="AD24" s="29" t="n">
         <f aca="false">SUM(AD18:AD23)</f>
-        <v>124691.02459894</v>
+        <v>123756.880697302</v>
       </c>
       <c r="AE24" s="29" t="n">
         <f aca="false">SUM(AE18:AE23)</f>
-        <v>140500.141002661</v>
+        <v>139483.773899232</v>
       </c>
       <c r="AF24" s="29" t="n">
         <f aca="false">SUM(AF18:AF23)</f>
-        <v>148369.740857785</v>
+        <v>147264.759988664</v>
       </c>
       <c r="AG24" s="29" t="n">
         <f aca="false">SUM(AG18:AG23)</f>
-        <v>165345.268986946</v>
+        <v>164144.767860812</v>
       </c>
       <c r="AH24" s="29" t="n">
         <f aca="false">SUM(AH18:AH23)</f>
-        <v>174475.790644926</v>
+        <v>173172.305685906</v>
       </c>
       <c r="AI24" s="29" t="n">
         <f aca="false">SUM(AI18:AI23)</f>
-        <v>192814.281532068</v>
+        <v>191399.747627102</v>
       </c>
       <c r="AJ24" s="29" t="n">
         <f aca="false">SUM(AJ18:AJ23)</f>
-        <v>203417.940999294</v>
+        <v>201883.643486435</v>
       </c>
       <c r="AK24" s="29" t="n">
         <f aca="false">SUM(AK18:AK23)</f>
-        <v>223348.530300281</v>
+        <v>221685.053113286</v>
       </c>
       <c r="AL24" s="29" t="n">
         <f aca="false">SUM(AL18:AL23)</f>
-        <v>244172.737894821</v>
+        <v>242369.907556587</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="14" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="C25" s="29" t="n">
         <f aca="false">C16-C24</f>
@@ -7652,128 +7751,128 @@
       </c>
       <c r="I25" s="29" t="n">
         <f aca="false">I16-I24</f>
-        <v>1386.8374</v>
+        <v>-1235.7365</v>
       </c>
       <c r="J25" s="29" t="n">
         <f aca="false">J16-J24</f>
-        <v>9533.368357</v>
+        <v>6274.1102425</v>
       </c>
       <c r="K25" s="29" t="n">
         <f aca="false">K16-K24</f>
-        <v>18153.632191435</v>
+        <v>14217.4270828375</v>
       </c>
       <c r="L25" s="29" t="n">
         <f aca="false">L16-L24</f>
-        <v>27289.9772734779</v>
+        <v>22633.0745698786</v>
       </c>
       <c r="M25" s="29" t="n">
         <f aca="false">M16-M24</f>
-        <v>36988.0285994161</v>
+        <v>31562.9175228726</v>
       </c>
       <c r="N25" s="29" t="n">
         <f aca="false">N16-N24</f>
-        <v>47296.9527028278</v>
+        <v>41052.067987421</v>
       </c>
       <c r="O25" s="29" t="n">
         <f aca="false">O16-O24</f>
-        <v>58269.743689126</v>
+        <v>51149.1475625653</v>
       </c>
       <c r="P25" s="29" t="n">
         <f aca="false">P16-P24</f>
-        <v>69963.5320850763</v>
+        <v>61906.5706503175</v>
       </c>
       <c r="Q25" s="29" t="n">
         <f aca="false">Q16-Q24</f>
-        <v>73939.918330182</v>
+        <v>64880.8503030211</v>
       </c>
       <c r="R25" s="29" t="n">
         <f aca="false">R16-R24</f>
-        <v>87265.3328829388</v>
+        <v>77132.928477924</v>
       </c>
       <c r="S25" s="29" t="n">
         <f aca="false">S16-S24</f>
-        <v>101511.425072757</v>
+        <v>90228.5326530527</v>
       </c>
       <c r="T25" s="29" t="n">
         <f aca="false">T16-T24</f>
-        <v>116755.482998782</v>
+        <v>104238.560914769</v>
       </c>
       <c r="U25" s="29" t="n">
         <f aca="false">U16-U24</f>
-        <v>133080.886960884</v>
+        <v>119239.497796186</v>
       </c>
       <c r="V25" s="29" t="n">
         <f aca="false">V16-V24</f>
-        <v>142077.599106898</v>
+        <v>126813.863327911</v>
       </c>
       <c r="W25" s="29" t="n">
         <f aca="false">W16-W24</f>
-        <v>160842.692194865</v>
+        <v>144050.697959473</v>
       </c>
       <c r="X25" s="29" t="n">
         <f aca="false">X16-X24</f>
-        <v>180980.920600885</v>
+        <v>162546.086222426</v>
       </c>
       <c r="Y25" s="29" t="n">
         <f aca="false">Y16-Y24</f>
-        <v>202605.336953625</v>
+        <v>182403.722235761</v>
       </c>
       <c r="Z25" s="29" t="n">
         <f aca="false">Z16-Z24</f>
-        <v>217337.958046967</v>
+        <v>195235.520402274</v>
       </c>
       <c r="AA25" s="29" t="n">
         <f aca="false">AA16-AA24</f>
-        <v>242310.483974351</v>
+        <v>218162.274912417</v>
       </c>
       <c r="AB25" s="29" t="n">
         <f aca="false">AB16-AB24</f>
-        <v>269165.074743834</v>
+        <v>242814.371961423</v>
       </c>
       <c r="AC25" s="29" t="n">
         <f aca="false">AC16-AC24</f>
-        <v>289555.188973588</v>
+        <v>260832.558897948</v>
       </c>
       <c r="AD25" s="29" t="n">
         <f aca="false">AD16-AD24</f>
-        <v>320646.489635466</v>
+        <v>289368.774859905</v>
       </c>
       <c r="AE25" s="29" t="n">
         <f aca="false">AE16-AE24</f>
-        <v>345617.822211695</v>
+        <v>311587.047817566</v>
       </c>
       <c r="AF25" s="29" t="n">
         <f aca="false">AF16-AF24</f>
-        <v>381662.271058887</v>
+        <v>344664.463337618</v>
       </c>
       <c r="AG25" s="29" t="n">
         <f aca="false">AG16-AG24</f>
-        <v>411988.300237098</v>
+        <v>371792.210806908</v>
       </c>
       <c r="AH25" s="29" t="n">
         <f aca="false">AH16-AH24</f>
-        <v>453820.985562228</v>
+        <v>410176.713313684</v>
       </c>
       <c r="AI25" s="29" t="n">
         <f aca="false">AI16-AI24</f>
-        <v>490403.345180715</v>
+        <v>443040.847879947</v>
       </c>
       <c r="AJ25" s="29" t="n">
         <f aca="false">AJ16-AJ24</f>
-        <v>538997.776549343</v>
+        <v>487625.263273981</v>
       </c>
       <c r="AK25" s="29" t="n">
         <f aca="false">AK16-AK24</f>
-        <v>582887.608333607</v>
+        <v>527189.803210448</v>
       </c>
       <c r="AL25" s="29" t="n">
         <f aca="false">AL16-AL24</f>
-        <v>630878.776419104</v>
+        <v>570515.043369968</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="C26" s="13" t="n">
         <f aca="false">IFERROR(C25/C16,0)</f>
@@ -7801,277 +7900,277 @@
       </c>
       <c r="I26" s="13" t="n">
         <f aca="false">IFERROR(I25/I16,0)</f>
-        <v>0.0943754227657215</v>
+        <v>-0.103029556444889</v>
       </c>
       <c r="J26" s="13" t="n">
         <f aca="false">IFERROR(J25/J16,0)</f>
-        <v>0.386898026115074</v>
+        <v>0.294781705743115</v>
       </c>
       <c r="K26" s="13" t="n">
         <f aca="false">IFERROR(K25/K16,0)</f>
-        <v>0.516277643475576</v>
+        <v>0.457023065764235</v>
       </c>
       <c r="L26" s="13" t="n">
         <f aca="false">IFERROR(L25/L16,0)</f>
-        <v>0.589256654588497</v>
+        <v>0.545157727087818</v>
       </c>
       <c r="M26" s="13" t="n">
         <f aca="false">IFERROR(M25/M16,0)</f>
-        <v>0.636121885024351</v>
+        <v>0.600523597368557</v>
       </c>
       <c r="N26" s="13" t="n">
         <f aca="false">IFERROR(N25/N16,0)</f>
-        <v>0.668761559715518</v>
+        <v>0.638527300921731</v>
       </c>
       <c r="O26" s="13" t="n">
         <f aca="false">IFERROR(O25/O16,0)</f>
-        <v>0.692794366341054</v>
+        <v>0.666221212592805</v>
       </c>
       <c r="P26" s="13" t="n">
         <f aca="false">IFERROR(P25/P16,0)</f>
-        <v>0.711221135874809</v>
+        <v>0.687290221823941</v>
       </c>
       <c r="Q26" s="13" t="n">
         <f aca="false">IFERROR(Q25/Q16,0)</f>
-        <v>0.650957621187896</v>
+        <v>0.622317978484784</v>
       </c>
       <c r="R26" s="13" t="n">
         <f aca="false">IFERROR(R25/R16,0)</f>
-        <v>0.672123077352728</v>
+        <v>0.646002657565962</v>
       </c>
       <c r="S26" s="13" t="n">
         <f aca="false">IFERROR(S25/S16,0)</f>
-        <v>0.689591383600815</v>
+        <v>0.665474235007907</v>
       </c>
       <c r="T26" s="13" t="n">
         <f aca="false">IFERROR(T25/T16,0)</f>
-        <v>0.704237064117516</v>
+        <v>0.681746601837938</v>
       </c>
       <c r="U26" s="13" t="n">
         <f aca="false">IFERROR(U25/U16,0)</f>
-        <v>0.716677506586945</v>
+        <v>0.695530860904023</v>
       </c>
       <c r="V26" s="13" t="n">
         <f aca="false">IFERROR(V25/V16,0)</f>
-        <v>0.68630210587612</v>
+        <v>0.662907690927283</v>
       </c>
       <c r="W26" s="13" t="n">
         <f aca="false">IFERROR(W25/W16,0)</f>
-        <v>0.699647576322019</v>
+        <v>0.677574717902409</v>
       </c>
       <c r="X26" s="13" t="n">
         <f aca="false">IFERROR(X25/X16,0)</f>
-        <v>0.711305143401699</v>
+        <v>0.690364721297607</v>
       </c>
       <c r="Y26" s="13" t="n">
         <f aca="false">IFERROR(Y25/Y16,0)</f>
-        <v>0.721558079526354</v>
+        <v>0.70159671855683</v>
       </c>
       <c r="Z26" s="13" t="n">
         <f aca="false">IFERROR(Z25/Z16,0)</f>
-        <v>0.703129996810599</v>
+        <v>0.681835575143933</v>
       </c>
       <c r="AA26" s="13" t="n">
         <f aca="false">IFERROR(AA25/AA16,0)</f>
-        <v>0.713661452404956</v>
+        <v>0.693322609040598</v>
       </c>
       <c r="AB26" s="13" t="n">
         <f aca="false">IFERROR(AB25/AB16,0)</f>
-        <v>0.723068226923906</v>
+        <v>0.70357249155702</v>
       </c>
       <c r="AC26" s="13" t="n">
         <f aca="false">IFERROR(AC25/AC16,0)</f>
-        <v>0.710642506290248</v>
+        <v>0.690261441515985</v>
       </c>
       <c r="AD26" s="13" t="n">
         <f aca="false">IFERROR(AD25/AD16,0)</f>
-        <v>0.720007812920723</v>
+        <v>0.700437677901211</v>
       </c>
       <c r="AE26" s="13" t="n">
         <f aca="false">IFERROR(AE25/AE16,0)</f>
-        <v>0.710975212531475</v>
+        <v>0.690771898372078</v>
       </c>
       <c r="AF26" s="13" t="n">
         <f aca="false">IFERROR(AF25/AF16,0)</f>
-        <v>0.720074000207537</v>
+        <v>0.700638317453673</v>
       </c>
       <c r="AG26" s="13" t="n">
         <f aca="false">IFERROR(AG25/AG16,0)</f>
-        <v>0.713605309302947</v>
+        <v>0.693723750376662</v>
       </c>
       <c r="AH26" s="13" t="n">
         <f aca="false">IFERROR(AH25/AH16,0)</f>
-        <v>0.722303539900068</v>
+        <v>0.703141172701573</v>
       </c>
       <c r="AI26" s="13" t="n">
         <f aca="false">IFERROR(AI25/AI16,0)</f>
-        <v>0.717784972176772</v>
+        <v>0.698317306643762</v>
       </c>
       <c r="AJ26" s="13" t="n">
         <f aca="false">IFERROR(AJ25/AJ16,0)</f>
-        <v>0.726005341493908</v>
+        <v>0.707206619802833</v>
       </c>
       <c r="AK26" s="13" t="n">
         <f aca="false">IFERROR(AK25/AK16,0)</f>
-        <v>0.722973804326447</v>
+        <v>0.703975836227764</v>
       </c>
       <c r="AL26" s="13" t="n">
         <f aca="false">IFERROR(AL25/AL16,0)</f>
-        <v>0.720961870357699</v>
+        <v>0.70183983935202</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="C28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=C4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=C4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=C4)*Staffing!$E$5:$E$15))</f>
         <v>61500</v>
       </c>
       <c r="D28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=D4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=D4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=D4)*Staffing!$E$5:$E$15))</f>
         <v>61500</v>
       </c>
       <c r="E28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=E4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=E4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=E4)*Staffing!$E$5:$E$15))</f>
         <v>61500</v>
       </c>
       <c r="F28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=F4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=F4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=F4)*Staffing!$E$5:$E$15))</f>
         <v>80500</v>
       </c>
       <c r="G28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=G4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=G4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=G4)*Staffing!$E$5:$E$15))</f>
         <v>80500</v>
       </c>
       <c r="H28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=H4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=H4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=H4)*Staffing!$E$5:$E$15))</f>
         <v>80500</v>
       </c>
       <c r="I28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=I4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=I4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=I4)*Staffing!$E$5:$E$15))</f>
         <v>93500</v>
       </c>
       <c r="J28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=J4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=J4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=J4)*Staffing!$E$5:$E$15))</f>
         <v>93500</v>
       </c>
       <c r="K28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=K4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=K4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=K4)*Staffing!$E$5:$E$15))</f>
         <v>93500</v>
       </c>
       <c r="L28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=L4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=L4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=L4)*Staffing!$E$5:$E$15))</f>
         <v>104500</v>
       </c>
       <c r="M28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=M4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=M4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=M4)*Staffing!$E$5:$E$15))</f>
         <v>104500</v>
       </c>
       <c r="N28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=N4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=N4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=N4)*Staffing!$E$5:$E$15))</f>
         <v>104500</v>
       </c>
       <c r="O28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=O4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=O4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=O4)*Staffing!$E$5:$E$15))</f>
         <v>122500</v>
       </c>
       <c r="P28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=P4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=P4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=P4)*Staffing!$E$5:$E$15))</f>
         <v>122500</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=Q4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=Q4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=Q4)*Staffing!$E$5:$E$15))</f>
         <v>122500</v>
       </c>
       <c r="R28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=R4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=R4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=R4)*Staffing!$E$5:$E$15))</f>
         <v>147500</v>
       </c>
       <c r="S28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=S4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=S4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=S4)*Staffing!$E$5:$E$15))</f>
         <v>147500</v>
       </c>
       <c r="T28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=T4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=T4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=T4)*Staffing!$E$5:$E$15))</f>
         <v>147500</v>
       </c>
       <c r="U28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=U4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=U4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=U4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="V28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=V4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=V4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=V4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="W28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=W4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=W4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=W4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="X28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=X4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=X4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=X4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="Y28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=Y4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=Y4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=Y4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="Z28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=Z4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=Z4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=Z4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AA28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AA4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AA4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AA4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AB28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AB4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AB4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AB4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AC28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AC4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AC4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AC4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AD28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AD4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AD4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AD4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AE28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AE4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AE4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AE4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AF28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AF4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AF4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AF4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AG28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AG4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AG4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AG4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AH28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AH4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AH4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AH4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AI4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AI4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AI4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AJ28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AJ4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AJ4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AJ4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AK28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AK4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AK4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AK4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
       <c r="AL28" s="6" t="n">
-        <f aca="false">SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AL4)*Staffing!$C$5:$C$15)</f>
+        <f aca="false">IF(Assumptions!$F$34=1,SUMPRODUCT((Staffing!$D$5:$D$15&lt;=AL4)*Staffing!$C$5:$C$15),SUMPRODUCT((Staffing!$F$5:$F$15&lt;=AL4)*Staffing!$E$5:$E$15))</f>
         <v>165500</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="C29" s="6" t="n">
         <f aca="false">C9*Assumptions!$F$21+IF(C4&gt;=Assumptions!$F$7-2,Assumptions!$F$25,0)</f>
@@ -8220,7 +8319,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="2" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C30" s="6" t="n">
         <f aca="false">Infrastructure!$C$28</f>
@@ -8369,7 +8468,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="C31" s="6" t="n">
         <f aca="false">Assumptions!$F$30</f>
@@ -8518,7 +8617,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="2" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="C32" s="6" t="n">
         <f aca="false">Assumptions!$F$31</f>
@@ -8667,7 +8766,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C33" s="6" t="n">
         <f aca="false">IF(C4&gt;=Assumptions!$F$33,Assumptions!$F$32,0)</f>
@@ -8816,156 +8915,156 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="2" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="D34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="E34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="F34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="G34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="H34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="I34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="J34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="K34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="L34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="M34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="N34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="O34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="P34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="R34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="S34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="T34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="U34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="V34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="W34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="X34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="Y34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="Z34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AA34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AB34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AC34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AD34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AE34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AF34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AG34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AH34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AI34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AJ34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AK34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
       <c r="AL34" s="6" t="n">
-        <f aca="false">Assumptions!$F$34</f>
+        <f aca="false">Assumptions!$F$35</f>
         <v>3000</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="2" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C35" s="6" t="n">
         <f aca="false">SUMIF(Setup!$D$5:$D$17,C4,Setup!$C$5:$C$17)</f>
@@ -9114,7 +9213,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="14" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="C36" s="29" t="n">
         <f aca="false">SUM(C28:C35)</f>
@@ -9263,7 +9362,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="14" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="C38" s="29" t="n">
         <f aca="false">C25-C36</f>
@@ -9291,128 +9390,128 @@
       </c>
       <c r="I38" s="29" t="n">
         <f aca="false">I25-I36</f>
-        <v>-134913.1626</v>
+        <v>-137535.7365</v>
       </c>
       <c r="J38" s="29" t="n">
         <f aca="false">J25-J36</f>
-        <v>-128686.631643</v>
+        <v>-131945.8897575</v>
       </c>
       <c r="K38" s="29" t="n">
         <f aca="false">K25-K36</f>
-        <v>-122139.967808565</v>
+        <v>-126076.172917163</v>
       </c>
       <c r="L38" s="29" t="n">
         <f aca="false">L25-L36</f>
-        <v>-126243.110726522</v>
+        <v>-130900.013430121</v>
       </c>
       <c r="M38" s="29" t="n">
         <f aca="false">M25-M36</f>
-        <v>-118963.706440584</v>
+        <v>-124388.817517127</v>
       </c>
       <c r="N38" s="29" t="n">
         <f aca="false">N25-N36</f>
-        <v>-111266.921140372</v>
+        <v>-117511.805855779</v>
       </c>
       <c r="O38" s="29" t="n">
         <f aca="false">O25-O36</f>
-        <v>-126115.24006153</v>
+        <v>-133235.836188091</v>
       </c>
       <c r="P38" s="29" t="n">
         <f aca="false">P25-P36</f>
-        <v>-117468.250365632</v>
+        <v>-125525.211800391</v>
       </c>
       <c r="Q38" s="29" t="n">
         <f aca="false">Q25-Q36</f>
-        <v>-116782.406716583</v>
+        <v>-125841.474743744</v>
       </c>
       <c r="R38" s="29" t="n">
         <f aca="false">R25-R36</f>
-        <v>-132010.778167568</v>
+        <v>-142143.182572582</v>
       </c>
       <c r="S38" s="29" t="n">
         <f aca="false">S25-S36</f>
-        <v>-121602.774861789</v>
+        <v>-132885.667281494</v>
       </c>
       <c r="T38" s="29" t="n">
         <f aca="false">T25-T36</f>
-        <v>-110503.852930529</v>
+        <v>-123020.775014541</v>
       </c>
       <c r="U38" s="29" t="n">
         <f aca="false">U25-U36</f>
-        <v>-116655.195842772</v>
+        <v>-130496.585007469</v>
       </c>
       <c r="V38" s="29" t="n">
         <f aca="false">V25-V36</f>
-        <v>-112493.37032105</v>
+        <v>-127757.106100037</v>
       </c>
       <c r="W38" s="29" t="n">
         <f aca="false">W25-W36</f>
-        <v>-98949.9547873183</v>
+        <v>-115741.949022711</v>
       </c>
       <c r="X38" s="29" t="n">
         <f aca="false">X25-X36</f>
-        <v>-84451.1381398739</v>
+        <v>-102885.972518332</v>
       </c>
       <c r="Y38" s="29" t="n">
         <f aca="false">Y25-Y36</f>
-        <v>-68917.2864863945</v>
+        <v>-89118.9012042581</v>
       </c>
       <c r="Z38" s="29" t="n">
         <f aca="false">Z25-Z36</f>
-        <v>-60762.4752682537</v>
+        <v>-82864.9129129464</v>
       </c>
       <c r="AA38" s="29" t="n">
         <f aca="false">AA25-AA36</f>
-        <v>-42893.9840060878</v>
+        <v>-67042.1930680212</v>
       </c>
       <c r="AB38" s="29" t="n">
         <f aca="false">AB25-AB36</f>
-        <v>-23711.7506750392</v>
+        <v>-50062.4534574509</v>
       </c>
       <c r="AC38" s="29" t="n">
         <f aca="false">AC25-AC36</f>
-        <v>-11607.7824787951</v>
+        <v>-40330.4125544352</v>
       </c>
       <c r="AD38" s="29" t="n">
         <f aca="false">AD25-AD36</f>
-        <v>10534.4804668923</v>
+        <v>-20743.2343086686</v>
       </c>
       <c r="AE38" s="29" t="n">
         <f aca="false">AE25-AE36</f>
-        <v>25840.8523096349</v>
+        <v>-8189.9220844938</v>
       </c>
       <c r="AF38" s="29" t="n">
         <f aca="false">AF25-AF36</f>
-        <v>51447.1435646621</v>
+        <v>14449.3358433933</v>
       </c>
       <c r="AG38" s="29" t="n">
         <f aca="false">AG25-AG36</f>
-        <v>70499.962543335</v>
+        <v>30303.8731131454</v>
       </c>
       <c r="AH38" s="29" t="n">
         <f aca="false">AH25-AH36</f>
-        <v>100157.580852964</v>
+        <v>56513.3086044203</v>
       </c>
       <c r="AI38" s="29" t="n">
         <f aca="false">AI25-AI36</f>
-        <v>123590.86809471</v>
+        <v>76228.370793942</v>
       </c>
       <c r="AJ38" s="29" t="n">
         <f aca="false">AJ25-AJ36</f>
-        <v>157984.301296458</v>
+        <v>106611.788021096</v>
       </c>
       <c r="AK38" s="29" t="n">
         <f aca="false">AK25-AK36</f>
-        <v>186537.055060491</v>
+        <v>130839.249937331</v>
       </c>
       <c r="AL38" s="29" t="n">
         <f aca="false">AL25-AL36</f>
-        <v>217964.178884139</v>
+        <v>157600.445835002</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="14" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="C39" s="29" t="n">
         <f aca="false">C38</f>
@@ -9440,128 +9539,128 @@
       </c>
       <c r="I39" s="29" t="n">
         <f aca="false">H39+I38</f>
-        <v>-874163.1626</v>
+        <v>-876785.7365</v>
       </c>
       <c r="J39" s="29" t="n">
         <f aca="false">I39+J38</f>
-        <v>-1002849.794243</v>
+        <v>-1008731.6262575</v>
       </c>
       <c r="K39" s="29" t="n">
         <f aca="false">J39+K38</f>
-        <v>-1124989.76205157</v>
+        <v>-1134807.79917466</v>
       </c>
       <c r="L39" s="29" t="n">
         <f aca="false">K39+L38</f>
-        <v>-1251232.87277809</v>
+        <v>-1265707.81260478</v>
       </c>
       <c r="M39" s="29" t="n">
         <f aca="false">L39+M38</f>
-        <v>-1370196.57921867</v>
+        <v>-1390096.63012191</v>
       </c>
       <c r="N39" s="29" t="n">
         <f aca="false">M39+N38</f>
-        <v>-1481463.50035904</v>
+        <v>-1507608.43597769</v>
       </c>
       <c r="O39" s="29" t="n">
         <f aca="false">N39+O38</f>
-        <v>-1607578.74042057</v>
+        <v>-1640844.27216578</v>
       </c>
       <c r="P39" s="29" t="n">
         <f aca="false">O39+P38</f>
-        <v>-1725046.99078621</v>
+        <v>-1766369.48396617</v>
       </c>
       <c r="Q39" s="29" t="n">
         <f aca="false">P39+Q38</f>
-        <v>-1841829.39750279</v>
+        <v>-1892210.95870992</v>
       </c>
       <c r="R39" s="29" t="n">
         <f aca="false">Q39+R38</f>
-        <v>-1973840.17567036</v>
+        <v>-2034354.1412825</v>
       </c>
       <c r="S39" s="29" t="n">
         <f aca="false">R39+S38</f>
-        <v>-2095442.95053215</v>
+        <v>-2167239.80856399</v>
       </c>
       <c r="T39" s="29" t="n">
         <f aca="false">S39+T38</f>
-        <v>-2205946.80346267</v>
+        <v>-2290260.58357853</v>
       </c>
       <c r="U39" s="29" t="n">
         <f aca="false">T39+U38</f>
-        <v>-2322601.99930545</v>
+        <v>-2420757.168586</v>
       </c>
       <c r="V39" s="29" t="n">
         <f aca="false">U39+V38</f>
-        <v>-2435095.3696265</v>
+        <v>-2548514.27468604</v>
       </c>
       <c r="W39" s="29" t="n">
         <f aca="false">V39+W38</f>
-        <v>-2534045.32441381</v>
+        <v>-2664256.22370875</v>
       </c>
       <c r="X39" s="29" t="n">
         <f aca="false">W39+X38</f>
-        <v>-2618496.46255369</v>
+        <v>-2767142.19622708</v>
       </c>
       <c r="Y39" s="29" t="n">
         <f aca="false">X39+Y38</f>
-        <v>-2687413.74904008</v>
+        <v>-2856261.09743134</v>
       </c>
       <c r="Z39" s="29" t="n">
         <f aca="false">Y39+Z38</f>
-        <v>-2748176.22430834</v>
+        <v>-2939126.01034429</v>
       </c>
       <c r="AA39" s="29" t="n">
         <f aca="false">Z39+AA38</f>
-        <v>-2791070.20831442</v>
+        <v>-3006168.20341231</v>
       </c>
       <c r="AB39" s="29" t="n">
         <f aca="false">AA39+AB38</f>
-        <v>-2814781.95898946</v>
+        <v>-3056230.65686976</v>
       </c>
       <c r="AC39" s="29" t="n">
         <f aca="false">AB39+AC38</f>
-        <v>-2826389.74146826</v>
+        <v>-3096561.0694242</v>
       </c>
       <c r="AD39" s="29" t="n">
         <f aca="false">AC39+AD38</f>
-        <v>-2815855.26100137</v>
+        <v>-3117304.30373286</v>
       </c>
       <c r="AE39" s="29" t="n">
         <f aca="false">AD39+AE38</f>
-        <v>-2790014.40869173</v>
+        <v>-3125494.22581736</v>
       </c>
       <c r="AF39" s="29" t="n">
         <f aca="false">AE39+AF38</f>
-        <v>-2738567.26512707</v>
+        <v>-3111044.88997396</v>
       </c>
       <c r="AG39" s="29" t="n">
         <f aca="false">AF39+AG38</f>
-        <v>-2668067.30258373</v>
+        <v>-3080741.01686082</v>
       </c>
       <c r="AH39" s="29" t="n">
         <f aca="false">AG39+AH38</f>
-        <v>-2567909.72173077</v>
+        <v>-3024227.7082564</v>
       </c>
       <c r="AI39" s="29" t="n">
         <f aca="false">AH39+AI38</f>
-        <v>-2444318.85363606</v>
+        <v>-2947999.33746246</v>
       </c>
       <c r="AJ39" s="29" t="n">
         <f aca="false">AI39+AJ38</f>
-        <v>-2286334.5523396</v>
+        <v>-2841387.54944136</v>
       </c>
       <c r="AK39" s="29" t="n">
         <f aca="false">AJ39+AK38</f>
-        <v>-2099797.49727911</v>
+        <v>-2710548.29950403</v>
       </c>
       <c r="AL39" s="29" t="n">
         <f aca="false">AK39+AL38</f>
-        <v>-1881833.31839497</v>
+        <v>-2552947.85366903</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="2" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="C40" s="6" t="n">
         <f aca="false">C24+C36</f>
@@ -9589,128 +9688,128 @@
       </c>
       <c r="I40" s="6" t="n">
         <f aca="false">I24+I36</f>
-        <v>149608.0626</v>
+        <v>149529.7365</v>
       </c>
       <c r="J40" s="6" t="n">
         <f aca="false">J24+J36</f>
-        <v>153327.151143</v>
+        <v>153229.8097575</v>
       </c>
       <c r="K40" s="6" t="n">
         <f aca="false">K24+K36</f>
-        <v>157302.505681065</v>
+        <v>157184.946517163</v>
       </c>
       <c r="L40" s="6" t="n">
         <f aca="false">L24+L36</f>
-        <v>172555.65902101</v>
+        <v>172416.575418121</v>
       </c>
       <c r="M40" s="6" t="n">
         <f aca="false">M24+M36</f>
-        <v>177109.840806013</v>
+        <v>176947.813801667</v>
       </c>
       <c r="N40" s="6" t="n">
         <f aca="false">N24+N36</f>
-        <v>181990.113907234</v>
+        <v>181803.603447145</v>
       </c>
       <c r="O40" s="6" t="n">
         <f aca="false">O24+O36</f>
-        <v>210223.521710634</v>
+        <v>210010.857150727</v>
       </c>
       <c r="P40" s="6" t="n">
         <f aca="false">P24+P36</f>
-        <v>215839.247171036</v>
+        <v>215598.6170149</v>
       </c>
       <c r="Q40" s="6" t="n">
         <f aca="false">Q24+Q36</f>
-        <v>230368.784575181</v>
+        <v>230098.225385904</v>
       </c>
       <c r="R40" s="6" t="n">
         <f aca="false">R24+R36</f>
-        <v>261846.125030896</v>
+        <v>261543.509451343</v>
       </c>
       <c r="S40" s="6" t="n">
         <f aca="false">S24+S36</f>
-        <v>268807.956780825</v>
+        <v>268470.980591153</v>
       </c>
       <c r="T40" s="6" t="n">
         <f aca="false">T24+T36</f>
-        <v>276293.881527063</v>
+        <v>275920.049662556</v>
       </c>
       <c r="U40" s="6" t="n">
         <f aca="false">U24+U36</f>
-        <v>302346.648047905</v>
+        <v>301933.259494067</v>
       </c>
       <c r="V40" s="6" t="n">
         <f aca="false">V24+V36</f>
-        <v>319512.404490448</v>
+        <v>319056.535965637</v>
       </c>
       <c r="W40" s="6" t="n">
         <f aca="false">W24+W36</f>
-        <v>328840.970833426</v>
+        <v>328339.459162132</v>
       </c>
       <c r="X40" s="6" t="n">
         <f aca="false">X24+X36</f>
-        <v>338886.133134249</v>
+        <v>338335.556206365</v>
       </c>
       <c r="Y40" s="6" t="n">
         <f aca="false">Y24+Y36</f>
-        <v>349705.961303284</v>
+        <v>349102.617506355</v>
       </c>
       <c r="Z40" s="6" t="n">
         <f aca="false">Z24+Z36</f>
-        <v>369863.152287885</v>
+        <v>369203.038290257</v>
       </c>
       <c r="AA40" s="6" t="n">
         <f aca="false">AA24+AA36</f>
-        <v>382425.400699245</v>
+        <v>381704.187452287</v>
       </c>
       <c r="AB40" s="6" t="n">
         <f aca="false">AB24+AB36</f>
-        <v>395965.799077806</v>
+        <v>395178.805894809</v>
       </c>
       <c r="AC40" s="6" t="n">
         <f aca="false">AC24+AC36</f>
-        <v>419063.270168586</v>
+        <v>418205.436726574</v>
       </c>
       <c r="AD40" s="6" t="n">
         <f aca="false">AD24+AD36</f>
-        <v>434803.033767515</v>
+        <v>433868.889865876</v>
       </c>
       <c r="AE40" s="6" t="n">
         <f aca="false">AE24+AE36</f>
-        <v>460277.110904721</v>
+        <v>459260.743801292</v>
       </c>
       <c r="AF40" s="6" t="n">
         <f aca="false">AF24+AF36</f>
-        <v>478584.86835201</v>
+        <v>477479.887482888</v>
       </c>
       <c r="AG40" s="6" t="n">
         <f aca="false">AG24+AG36</f>
-        <v>506833.606680708</v>
+        <v>505633.105554575</v>
       </c>
       <c r="AH40" s="6" t="n">
         <f aca="false">AH24+AH36</f>
-        <v>528139.195354189</v>
+        <v>526835.71039517</v>
       </c>
       <c r="AI40" s="6" t="n">
         <f aca="false">AI24+AI36</f>
-        <v>559626.758618073</v>
+        <v>558212.224713107</v>
       </c>
       <c r="AJ40" s="6" t="n">
         <f aca="false">AJ24+AJ36</f>
-        <v>584431.416252179</v>
+        <v>582897.118739321</v>
       </c>
       <c r="AK40" s="6" t="n">
         <f aca="false">AK24+AK36</f>
-        <v>619699.083573397</v>
+        <v>618035.606386403</v>
       </c>
       <c r="AL40" s="6" t="n">
         <f aca="false">AL24+AL36</f>
-        <v>657087.335429786</v>
+        <v>655284.505091553</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="2" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C42" s="8" t="n">
         <f aca="false">IF(AND(C6=1,C38&gt;0),C4,999)</f>
@@ -9822,11 +9921,11 @@
       </c>
       <c r="AD42" s="8" t="n">
         <f aca="false">IF(AND(AD6=1,AD38&gt;0),AD4,999)</f>
-        <v>28</v>
+        <v>999</v>
       </c>
       <c r="AE42" s="8" t="n">
         <f aca="false">IF(AND(AE6=1,AE38&gt;0),AE4,999)</f>
-        <v>29</v>
+        <v>999</v>
       </c>
       <c r="AF42" s="8" t="n">
         <f aca="false">IF(AND(AF6=1,AF38&gt;0),AF4,999)</f>
@@ -9859,7 +9958,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="2" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C43" s="8" t="n">
         <f aca="false">IF(AND(C6=1,C39&gt;=0),C4,999)</f>

</xml_diff>